<commit_message>
운동프로그램 갱신 2026-10-02 16:15:28.99
</commit_message>
<xml_diff>
--- a/운동프로그램_주6회_v20.xlsx
+++ b/운동프로그램_주6회_v20.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b2bc197408547891/Desktop/운동/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_8E3F657BE93238B977D730997BA8BB14DC6B1CFA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="11_8E3F657BE93238B977D730997BA8BB14DC6B1CFA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA870588-3AAE-48BF-AC2C-A9BCFC049B84}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="976" firstSheet="1" activeTab="21" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="976" firstSheet="3" activeTab="23" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="시작중량_설정" sheetId="1" r:id="rId1"/>
@@ -8628,7 +8628,7 @@
         <v>4</v>
       </c>
       <c r="F71">
-        <f t="shared" ref="F71:F102" ca="1" si="4">IF(ISNUMBER(E71),$D71*E71,0)</f>
+        <f t="shared" ref="F71:F75" ca="1" si="4">IF(ISNUMBER(E71),$D71*E71,0)</f>
         <v>2</v>
       </c>
       <c r="G71" t="s">
@@ -11298,7 +11298,7 @@
       </c>
       <c r="E8" s="121">
         <f>복귀_월_가슴!$E$24</f>
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F8" s="114" t="s">
         <v>927</v>
@@ -11411,7 +11411,7 @@
       <c r="D13" s="122"/>
       <c r="E13" s="116">
         <f>SUM(E6:E12)</f>
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F13" s="116" t="s">
         <v>946</v>
@@ -13167,20 +13167,20 @@
         <v>35</v>
       </c>
       <c r="E18" s="112">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F18" s="112">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="G18" s="112">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="H18" s="112">
         <v>180</v>
       </c>
       <c r="I18" s="112">
         <f t="shared" ref="I18:I23" si="0">IF(E18=0,0,ROUND((E18*(G18+H18)+N18)/60,1))</f>
-        <v>17.5</v>
+        <v>15.3</v>
       </c>
       <c r="J18" s="113" t="s">
         <v>1084</v>
@@ -13400,14 +13400,14 @@
       </c>
       <c r="E24" s="116">
         <f>SUM(E18:E23)</f>
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F24" s="116"/>
       <c r="G24" s="116"/>
       <c r="H24" s="116"/>
       <c r="I24" s="116">
         <f>ROUND(SUM(I18:I23),0)</f>
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="26" spans="1:14">
@@ -16117,7 +16117,7 @@
         <v>10</v>
       </c>
       <c r="E18" s="114">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F18" s="114" t="s">
         <v>303</v>
@@ -16130,7 +16130,7 @@
       </c>
       <c r="I18" s="114">
         <f t="shared" si="0"/>
-        <v>10.7</v>
+        <v>8.3000000000000007</v>
       </c>
       <c r="J18" s="115" t="s">
         <v>1235</v>
@@ -16318,7 +16318,7 @@
         <v>297</v>
       </c>
       <c r="E23" s="114">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F23" s="114" t="s">
         <v>303</v>
@@ -16331,7 +16331,7 @@
       </c>
       <c r="I23" s="114">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>6.7</v>
       </c>
       <c r="J23" s="115" t="s">
         <v>1244</v>
@@ -16359,7 +16359,7 @@
       <c r="H24" s="116"/>
       <c r="I24" s="116">
         <f>ROUND(SUM(I11:I23),0)</f>
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="26" spans="1:14">
@@ -16933,11 +16933,11 @@
       </c>
       <c r="E7" s="114">
         <f t="shared" ref="E7:E38" ca="1" si="0">IFERROR(INDEX(INDIRECT("'"&amp;$A7&amp;"'!$E$1:$E$60"),MATCH($B7,INDIRECT("'"&amp;$A7&amp;"'!$B$1:$B$60"),0)),"?")</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F7" s="114">
         <f t="shared" ref="F7:F38" ca="1" si="1">IF(ISNUMBER(E7),$D7*E7,0)</f>
-        <v>1.6500000000000001</v>
+        <v>1.32</v>
       </c>
       <c r="G7" s="114" t="s">
         <v>673</v>
@@ -17269,11 +17269,11 @@
       </c>
       <c r="E19" s="114">
         <f t="shared" ca="1" si="0"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F19" s="114">
         <f t="shared" ca="1" si="1"/>
-        <v>1.6500000000000001</v>
+        <v>1.32</v>
       </c>
       <c r="G19" s="114" t="s">
         <v>673</v>
@@ -18529,7 +18529,7 @@
       </c>
       <c r="E64" s="114">
         <f t="shared" ca="1" si="2"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F64" s="114">
         <f t="shared" ca="1" si="3"/>
@@ -18788,7 +18788,7 @@
       </c>
       <c r="I5" s="125">
         <f ca="1">SUM(D5:D6)</f>
-        <v>25.5</v>
+        <v>23.5</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="30" customHeight="1">
@@ -18797,7 +18797,7 @@
       </c>
       <c r="B6" s="114">
         <f>SUMIFS(복귀_토_하체전면!$E:$E,복귀_토_하체전면!$C:$C,$A6)+SUMIFS(복귀_일_수평당기기!$E:$E,복귀_일_수평당기기!$C:$C,$A6)+SUMIFS(복귀_월_가슴!$E:$E,복귀_월_가슴!$C:$C,$A6)+SUMIFS(복귀_화_팔!$E:$E,복귀_화_팔!$C:$C,$A6)+SUMIFS(복귀_수_하체후면!$E:$E,복귀_수_하체후면!$C:$C,$A6)+SUMIFS(복귀_목_수직당기기!$E:$E,복귀_목_수직당기기!$C:$C,$A6)</f>
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C6" s="114">
         <f ca="1">MROUND(SUMIFS(복귀_간접계수맵!$F$7:$F$90,복귀_간접계수맵!$C$7:$C$90,$A6),0.5)</f>
@@ -18805,7 +18805,7 @@
       </c>
       <c r="D6" s="114">
         <f t="shared" ca="1" si="0"/>
-        <v>16.5</v>
+        <v>14.5</v>
       </c>
       <c r="E6" s="114" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -18931,7 +18931,7 @@
       </c>
       <c r="B11" s="114">
         <f>SUMIFS(복귀_토_하체전면!$E:$E,복귀_토_하체전면!$C:$C,$A11)+SUMIFS(복귀_일_수평당기기!$E:$E,복귀_일_수평당기기!$C:$C,$A11)+SUMIFS(복귀_월_가슴!$E:$E,복귀_월_가슴!$C:$C,$A11)+SUMIFS(복귀_화_팔!$E:$E,복귀_화_팔!$C:$C,$A11)+SUMIFS(복귀_수_하체후면!$E:$E,복귀_수_하체후면!$C:$C,$A11)+SUMIFS(복귀_목_수직당기기!$E:$E,복귀_목_수직당기기!$C:$C,$A11)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C11" s="114">
         <f ca="1">MROUND(SUMIFS(복귀_간접계수맵!$F$7:$F$90,복귀_간접계수맵!$C$7:$C$90,$A11),0.5)</f>
@@ -18939,7 +18939,7 @@
       </c>
       <c r="D11" s="114">
         <f t="shared" ca="1" si="0"/>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E11" s="114" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -19298,11 +19298,11 @@
       </c>
       <c r="B26" s="116">
         <f>SUM(B5:B25)</f>
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D26" s="116">
         <f ca="1">SUM(D5:D25)</f>
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="28" spans="1:6">

</xml_diff>

<commit_message>
운동프로그램 갱신 2026-10-04 23:02:21.04
</commit_message>
<xml_diff>
--- a/운동프로그램_주6회_v20.xlsx
+++ b/운동프로그램_주6회_v20.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b2bc197408547891/Desktop/운동/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="611" documentId="11_6AF0B42629B6F5CFF7DAC05DB27E968F34409905" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9B8FD4E2-A4BB-4FF2-86F6-D2FAD7D5439A}"/>
+  <xr:revisionPtr revIDLastSave="616" documentId="11_6AF0B42629B6F5CFF7DAC05DB27E968F34409905" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AE455280-6587-4AFB-9A7B-8867B4DC3081}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="976" firstSheet="1" activeTab="22" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="976" firstSheet="1" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="시작중량_설정" sheetId="1" r:id="rId1"/>
@@ -4326,144 +4326,6 @@
   </si>
   <si>
     <t>약 486분 (8시간 6분)</t>
-    <phoneticPr fontId="29" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">https://www.youtube.com/shorts/KGkE5bXQR24, </t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color theme="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-      </rPr>
-      <t>명치가</t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color theme="10"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color theme="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-      </rPr>
-      <t>의자</t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color theme="10"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color theme="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-      </rPr>
-      <t>최상단</t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color theme="10"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color theme="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-      </rPr>
-      <t>높이에</t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color theme="10"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color theme="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-      </rPr>
-      <t>맞게</t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color theme="10"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color theme="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="2"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">설정, </t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color theme="10"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t>https://www.youtube.com/shorts/W0TMqVIhpcQ</t>
-    </r>
     <phoneticPr fontId="29" type="noConversion"/>
   </si>
   <si>
@@ -5613,6 +5475,10 @@
   </si>
   <si>
     <t>· 기본은 증량 6주 + 디로드 1주(7주 덩어리)다 — 시작중량_설정 '디로드 간격(주)' = 7로 앱이 자동 반복한다(2026-10-04 사용자 지정: 10/17 · 12/5 · 1/23 · 3/13 …). 토요일 스쿼트가 2주 연속 안 오르면 그 시점에 앞당기고, 그 토요일을 '디로드 시작일'에 추가한다.</t>
+    <phoneticPr fontId="29" type="noConversion"/>
+  </si>
+  <si>
+    <t>당겼을 때 손잡이가 아래쪽 갈비뼈에서 명치 사이에 닿고, 팔꿈치는 몸통 옆을 지나 뒤로 빠져야 합니다., 패드는 가슴이 패드에서 떨어지지 않는 거리</t>
     <phoneticPr fontId="29" type="noConversion"/>
   </si>
 </sst>
@@ -6189,7 +6055,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="142">
+  <cellXfs count="143">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -6499,7 +6365,8 @@
     <xf numFmtId="49" fontId="58" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="58" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="57" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="22" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -6511,7 +6378,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="58" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -7486,24 +7353,24 @@
     </row>
     <row r="63" spans="1:5">
       <c r="A63" t="s">
-        <v>1486</v>
+        <v>1485</v>
       </c>
       <c r="C63" s="100">
         <v>46312</v>
       </c>
       <c r="D63" t="s">
-        <v>1492</v>
+        <v>1491</v>
       </c>
     </row>
     <row r="64" spans="1:5">
       <c r="A64" t="s">
+        <v>1489</v>
+      </c>
+      <c r="C64" s="135">
+        <v>7</v>
+      </c>
+      <c r="D64" t="s">
         <v>1490</v>
-      </c>
-      <c r="C64" s="141">
-        <v>7</v>
-      </c>
-      <c r="D64" t="s">
-        <v>1491</v>
       </c>
     </row>
     <row r="65" spans="1:4">
@@ -7534,7 +7401,7 @@
     </row>
     <row r="69" spans="1:4">
       <c r="A69" t="s">
-        <v>1487</v>
+        <v>1486</v>
       </c>
     </row>
     <row r="70" spans="1:4">
@@ -8241,16 +8108,16 @@
       </c>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1">
-      <c r="A2" s="138" t="s">
+      <c r="A2" s="139" t="s">
         <v>641</v>
       </c>
-      <c r="B2" s="137"/>
-      <c r="C2" s="137"/>
-      <c r="D2" s="137"/>
-      <c r="E2" s="137"/>
-      <c r="F2" s="137"/>
-      <c r="G2" s="137"/>
-      <c r="H2" s="137"/>
+      <c r="B2" s="138"/>
+      <c r="C2" s="138"/>
+      <c r="D2" s="138"/>
+      <c r="E2" s="138"/>
+      <c r="F2" s="138"/>
+      <c r="G2" s="138"/>
+      <c r="H2" s="138"/>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="s">
@@ -8262,16 +8129,16 @@
       </c>
     </row>
     <row r="4" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A4" s="136" t="s">
+      <c r="A4" s="137" t="s">
         <v>643</v>
       </c>
-      <c r="B4" s="137"/>
-      <c r="C4" s="137"/>
-      <c r="D4" s="137"/>
-      <c r="E4" s="137"/>
-      <c r="F4" s="137"/>
-      <c r="G4" s="137"/>
-      <c r="H4" s="137"/>
+      <c r="B4" s="138"/>
+      <c r="C4" s="138"/>
+      <c r="D4" s="138"/>
+      <c r="E4" s="138"/>
+      <c r="F4" s="138"/>
+      <c r="G4" s="138"/>
+      <c r="H4" s="138"/>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1">
       <c r="A6" s="44" t="s">
@@ -10361,7 +10228,7 @@
       <c r="F5" s="53" t="s">
         <v>744</v>
       </c>
-      <c r="G5" s="139" t="s">
+      <c r="G5" s="140" t="s">
         <v>745</v>
       </c>
       <c r="H5" s="56">
@@ -10404,7 +10271,7 @@
       <c r="F6" s="53" t="s">
         <v>746</v>
       </c>
-      <c r="G6" s="140"/>
+      <c r="G6" s="141"/>
       <c r="J6" s="55">
         <f t="shared" ca="1" si="2"/>
         <v>12.6</v>
@@ -10437,7 +10304,7 @@
       <c r="F7" s="53" t="s">
         <v>747</v>
       </c>
-      <c r="G7" s="139" t="s">
+      <c r="G7" s="140" t="s">
         <v>748</v>
       </c>
       <c r="H7" s="56">
@@ -10476,7 +10343,7 @@
       <c r="F8" s="53" t="s">
         <v>749</v>
       </c>
-      <c r="G8" s="140"/>
+      <c r="G8" s="141"/>
       <c r="J8" s="55">
         <f t="shared" ca="1" si="2"/>
         <v>3.9</v>
@@ -10509,7 +10376,7 @@
       <c r="F9" s="53" t="s">
         <v>750</v>
       </c>
-      <c r="G9" s="140"/>
+      <c r="G9" s="141"/>
       <c r="J9" s="55">
         <f t="shared" ca="1" si="2"/>
         <v>9.5</v>
@@ -10542,7 +10409,7 @@
       <c r="F10" s="53" t="s">
         <v>751</v>
       </c>
-      <c r="G10" s="140"/>
+      <c r="G10" s="141"/>
       <c r="J10" s="55">
         <f t="shared" ca="1" si="2"/>
         <v>14.4</v>
@@ -10780,7 +10647,7 @@
       <c r="F17" s="53" t="s">
         <v>758</v>
       </c>
-      <c r="G17" s="139" t="s">
+      <c r="G17" s="140" t="s">
         <v>382</v>
       </c>
       <c r="H17" s="56">
@@ -10819,7 +10686,7 @@
       <c r="F18" s="53" t="s">
         <v>759</v>
       </c>
-      <c r="G18" s="140"/>
+      <c r="G18" s="141"/>
       <c r="J18" s="55">
         <f t="shared" ca="1" si="2"/>
         <v>9.1</v>
@@ -12758,7 +12625,7 @@
         <v>32</v>
       </c>
       <c r="F7" s="114" t="s">
-        <v>1480</v>
+        <v>1479</v>
       </c>
       <c r="G7" s="115" t="s">
         <v>914</v>
@@ -12806,10 +12673,10 @@
         <v>24</v>
       </c>
       <c r="F9" s="114" t="s">
-        <v>1468</v>
+        <v>1467</v>
       </c>
       <c r="G9" s="115" t="s">
-        <v>1470</v>
+        <v>1469</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="30" customHeight="1">
@@ -12854,7 +12721,7 @@
         <v>43</v>
       </c>
       <c r="F11" s="114" t="s">
-        <v>1469</v>
+        <v>1468</v>
       </c>
       <c r="G11" s="115" t="s">
         <v>930</v>
@@ -13046,12 +12913,12 @@
     </row>
     <row r="45" spans="1:1">
       <c r="A45" s="126" t="s">
-        <v>1471</v>
+        <v>1470</v>
       </c>
     </row>
     <row r="46" spans="1:1">
       <c r="A46" s="126" t="s">
-        <v>1481</v>
+        <v>1480</v>
       </c>
     </row>
     <row r="47" spans="1:1">
@@ -13116,7 +12983,7 @@
     </row>
     <row r="61" spans="1:1">
       <c r="A61" s="123" t="s">
-        <v>1482</v>
+        <v>1481</v>
       </c>
     </row>
     <row r="62" spans="1:1">
@@ -14024,8 +13891,8 @@
         <f t="shared" si="0"/>
         <v>9.5</v>
       </c>
-      <c r="J12" s="75" t="s">
-        <v>1406</v>
+      <c r="J12" s="136" t="s">
+        <v>1493</v>
       </c>
       <c r="K12" s="115" t="s">
         <v>1026</v>
@@ -14306,7 +14173,7 @@
         <v>2.5</v>
       </c>
       <c r="J19" s="115" t="s">
-        <v>1475</v>
+        <v>1474</v>
       </c>
       <c r="K19" s="115" t="s">
         <v>1038</v>
@@ -15362,7 +15229,7 @@
         <v>0</v>
       </c>
       <c r="J14" s="115" t="s">
-        <v>1476</v>
+        <v>1475</v>
       </c>
       <c r="K14" s="115" t="s">
         <v>1038</v>
@@ -15646,12 +15513,12 @@
     </row>
     <row r="35" spans="1:1">
       <c r="A35" s="117" t="s">
-        <v>1473</v>
+        <v>1472</v>
       </c>
     </row>
     <row r="36" spans="1:1">
       <c r="A36" s="117" t="s">
-        <v>1474</v>
+        <v>1473</v>
       </c>
     </row>
     <row r="38" spans="1:1">
@@ -17841,7 +17708,7 @@
         <v>5.8</v>
       </c>
       <c r="J20" s="75" t="s">
-        <v>1407</v>
+        <v>1406</v>
       </c>
       <c r="K20" s="115" t="s">
         <v>1207</v>
@@ -17880,7 +17747,7 @@
         <v>1.7</v>
       </c>
       <c r="J21" s="115" t="s">
-        <v>1477</v>
+        <v>1476</v>
       </c>
       <c r="K21" s="115" t="s">
         <v>1038</v>
@@ -18123,17 +17990,17 @@
   <sheetData>
     <row r="1" spans="1:6" ht="18.75">
       <c r="A1" s="128" t="s">
-        <v>1408</v>
+        <v>1407</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="127" t="s">
-        <v>1409</v>
+        <v>1408</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="15">
       <c r="A4" s="99" t="s">
-        <v>1410</v>
+        <v>1409</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -18154,131 +18021,131 @@
       <c r="A6" s="127" t="s">
         <v>901</v>
       </c>
-      <c r="B6" s="135" t="s">
+      <c r="B6" s="142" t="s">
+        <v>1410</v>
+      </c>
+      <c r="C6" s="142"/>
+      <c r="D6" s="142"/>
+      <c r="E6" s="142"/>
+      <c r="F6" s="127" t="s">
         <v>1411</v>
-      </c>
-      <c r="C6" s="135"/>
-      <c r="D6" s="135"/>
-      <c r="E6" s="135"/>
-      <c r="F6" s="127" t="s">
-        <v>1412</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="127" t="s">
         <v>82</v>
       </c>
-      <c r="B7" s="135" t="s">
+      <c r="B7" s="142" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C7" s="142"/>
+      <c r="D7" s="142"/>
+      <c r="E7" s="142"/>
+      <c r="F7" s="127" t="s">
         <v>1413</v>
-      </c>
-      <c r="C7" s="135"/>
-      <c r="D7" s="135"/>
-      <c r="E7" s="135"/>
-      <c r="F7" s="127" t="s">
-        <v>1414</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="127" t="s">
+        <v>1414</v>
+      </c>
+      <c r="B8" s="142" t="s">
         <v>1415</v>
       </c>
-      <c r="B8" s="135" t="s">
+      <c r="C8" s="142"/>
+      <c r="D8" s="142"/>
+      <c r="E8" s="142"/>
+      <c r="F8" s="127" t="s">
         <v>1416</v>
-      </c>
-      <c r="C8" s="135"/>
-      <c r="D8" s="135"/>
-      <c r="E8" s="135"/>
-      <c r="F8" s="127" t="s">
-        <v>1417</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="127" t="s">
+        <v>1417</v>
+      </c>
+      <c r="B9" s="142" t="s">
         <v>1418</v>
       </c>
-      <c r="B9" s="135" t="s">
+      <c r="C9" s="142"/>
+      <c r="D9" s="142"/>
+      <c r="E9" s="142"/>
+      <c r="F9" s="127" t="s">
         <v>1419</v>
-      </c>
-      <c r="C9" s="135"/>
-      <c r="D9" s="135"/>
-      <c r="E9" s="135"/>
-      <c r="F9" s="127" t="s">
-        <v>1420</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="127" t="s">
+        <v>1420</v>
+      </c>
+      <c r="B10" s="142" t="s">
         <v>1421</v>
       </c>
-      <c r="B10" s="135" t="s">
-        <v>1422</v>
-      </c>
-      <c r="C10" s="135"/>
-      <c r="D10" s="135"/>
-      <c r="E10" s="135"/>
+      <c r="C10" s="142"/>
+      <c r="D10" s="142"/>
+      <c r="E10" s="142"/>
       <c r="F10" s="127" t="s">
-        <v>1485</v>
+        <v>1484</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="127" t="s">
+        <v>1422</v>
+      </c>
+      <c r="B11" s="142" t="s">
         <v>1423</v>
       </c>
-      <c r="B11" s="135" t="s">
+      <c r="C11" s="142"/>
+      <c r="D11" s="142"/>
+      <c r="E11" s="142"/>
+      <c r="F11" s="127" t="s">
         <v>1424</v>
-      </c>
-      <c r="C11" s="135"/>
-      <c r="D11" s="135"/>
-      <c r="E11" s="135"/>
-      <c r="F11" s="127" t="s">
-        <v>1425</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="127" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="135" t="s">
-        <v>1426</v>
-      </c>
-      <c r="C12" s="135"/>
-      <c r="D12" s="135"/>
-      <c r="E12" s="135"/>
+      <c r="B12" s="142" t="s">
+        <v>1425</v>
+      </c>
+      <c r="C12" s="142"/>
+      <c r="D12" s="142"/>
+      <c r="E12" s="142"/>
       <c r="F12" s="127" t="s">
-        <v>1467</v>
+        <v>1466</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="127" t="s">
+        <v>1426</v>
+      </c>
+      <c r="B13" s="142" t="s">
         <v>1427</v>
       </c>
-      <c r="B13" s="135" t="s">
-        <v>1428</v>
-      </c>
-      <c r="C13" s="135"/>
-      <c r="D13" s="135"/>
-      <c r="E13" s="135"/>
+      <c r="C13" s="142"/>
+      <c r="D13" s="142"/>
+      <c r="E13" s="142"/>
       <c r="F13" s="127" t="s">
-        <v>1484</v>
+        <v>1483</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="127" t="s">
+        <v>1428</v>
+      </c>
+      <c r="B14" s="142" t="s">
         <v>1429</v>
       </c>
-      <c r="B14" s="135" t="s">
+      <c r="C14" s="142"/>
+      <c r="D14" s="142"/>
+      <c r="E14" s="142"/>
+      <c r="F14" s="127" t="s">
         <v>1430</v>
-      </c>
-      <c r="C14" s="135"/>
-      <c r="D14" s="135"/>
-      <c r="E14" s="135"/>
-      <c r="F14" s="127" t="s">
-        <v>1431</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="15">
       <c r="A16" s="131" t="s">
-        <v>1432</v>
+        <v>1431</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -18286,19 +18153,19 @@
         <v>121</v>
       </c>
       <c r="B17" s="129" t="s">
+        <v>1432</v>
+      </c>
+      <c r="C17" s="129" t="s">
         <v>1433</v>
       </c>
-      <c r="C17" s="129" t="s">
+      <c r="D17" s="129" t="s">
         <v>1434</v>
       </c>
-      <c r="D17" s="129" t="s">
+      <c r="E17" s="129" t="s">
         <v>1435</v>
       </c>
-      <c r="E17" s="129" t="s">
+      <c r="F17" s="129" t="s">
         <v>1436</v>
-      </c>
-      <c r="F17" s="129" t="s">
-        <v>1437</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -18463,7 +18330,7 @@
     </row>
     <row r="28" spans="1:6">
       <c r="A28" s="127" t="s">
-        <v>1489</v>
+        <v>1488</v>
       </c>
     </row>
   </sheetData>
@@ -18498,12 +18365,12 @@
   <sheetData>
     <row r="1" spans="1:9" ht="18.75">
       <c r="A1" s="128" t="s">
-        <v>1466</v>
+        <v>1465</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" s="127" t="s">
-        <v>1438</v>
+        <v>1437</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="15">
@@ -18516,7 +18383,7 @@
         <v>901</v>
       </c>
       <c r="B5" s="129" t="s">
-        <v>1439</v>
+        <v>1438</v>
       </c>
       <c r="C5" s="130"/>
       <c r="D5" s="130"/>
@@ -18532,124 +18399,124 @@
       <c r="A6" s="127" t="s">
         <v>906</v>
       </c>
-      <c r="B6" s="135" t="s">
+      <c r="B6" s="142" t="s">
+        <v>1439</v>
+      </c>
+      <c r="C6" s="142"/>
+      <c r="D6" s="142"/>
+      <c r="E6" s="142"/>
+      <c r="F6" s="142"/>
+      <c r="G6" s="142"/>
+      <c r="H6" s="142"/>
+      <c r="I6" s="127" t="s">
         <v>1440</v>
-      </c>
-      <c r="C6" s="135"/>
-      <c r="D6" s="135"/>
-      <c r="E6" s="135"/>
-      <c r="F6" s="135"/>
-      <c r="G6" s="135"/>
-      <c r="H6" s="135"/>
-      <c r="I6" s="127" t="s">
-        <v>1441</v>
       </c>
     </row>
     <row r="7" spans="1:9">
       <c r="A7" s="127" t="s">
         <v>911</v>
       </c>
-      <c r="B7" s="135" t="s">
+      <c r="B7" s="142" t="s">
+        <v>1441</v>
+      </c>
+      <c r="C7" s="142"/>
+      <c r="D7" s="142"/>
+      <c r="E7" s="142"/>
+      <c r="F7" s="142"/>
+      <c r="G7" s="142"/>
+      <c r="H7" s="142"/>
+      <c r="I7" s="127" t="s">
         <v>1442</v>
-      </c>
-      <c r="C7" s="135"/>
-      <c r="D7" s="135"/>
-      <c r="E7" s="135"/>
-      <c r="F7" s="135"/>
-      <c r="G7" s="135"/>
-      <c r="H7" s="135"/>
-      <c r="I7" s="127" t="s">
-        <v>1443</v>
       </c>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" s="127" t="s">
         <v>915</v>
       </c>
-      <c r="B8" s="135" t="s">
+      <c r="B8" s="142" t="s">
+        <v>1441</v>
+      </c>
+      <c r="C8" s="142"/>
+      <c r="D8" s="142"/>
+      <c r="E8" s="142"/>
+      <c r="F8" s="142"/>
+      <c r="G8" s="142"/>
+      <c r="H8" s="142"/>
+      <c r="I8" s="127" t="s">
         <v>1442</v>
-      </c>
-      <c r="C8" s="135"/>
-      <c r="D8" s="135"/>
-      <c r="E8" s="135"/>
-      <c r="F8" s="135"/>
-      <c r="G8" s="135"/>
-      <c r="H8" s="135"/>
-      <c r="I8" s="127" t="s">
-        <v>1443</v>
       </c>
     </row>
     <row r="9" spans="1:9">
       <c r="A9" s="127" t="s">
         <v>919</v>
       </c>
-      <c r="B9" s="135" t="s">
+      <c r="B9" s="142" t="s">
         <v>29</v>
       </c>
-      <c r="C9" s="135"/>
-      <c r="D9" s="135"/>
-      <c r="E9" s="135"/>
-      <c r="F9" s="135"/>
-      <c r="G9" s="135"/>
-      <c r="H9" s="135"/>
+      <c r="C9" s="142"/>
+      <c r="D9" s="142"/>
+      <c r="E9" s="142"/>
+      <c r="F9" s="142"/>
+      <c r="G9" s="142"/>
+      <c r="H9" s="142"/>
       <c r="I9" s="127" t="s">
-        <v>1444</v>
+        <v>1443</v>
       </c>
     </row>
     <row r="10" spans="1:9">
       <c r="A10" s="127" t="s">
         <v>922</v>
       </c>
-      <c r="B10" s="135" t="s">
-        <v>1440</v>
-      </c>
-      <c r="C10" s="135"/>
-      <c r="D10" s="135"/>
-      <c r="E10" s="135"/>
-      <c r="F10" s="135"/>
-      <c r="G10" s="135"/>
-      <c r="H10" s="135"/>
+      <c r="B10" s="142" t="s">
+        <v>1439</v>
+      </c>
+      <c r="C10" s="142"/>
+      <c r="D10" s="142"/>
+      <c r="E10" s="142"/>
+      <c r="F10" s="142"/>
+      <c r="G10" s="142"/>
+      <c r="H10" s="142"/>
       <c r="I10" s="127" t="s">
-        <v>1445</v>
+        <v>1444</v>
       </c>
     </row>
     <row r="11" spans="1:9">
       <c r="A11" s="127" t="s">
         <v>927</v>
       </c>
-      <c r="B11" s="135" t="s">
+      <c r="B11" s="142" t="s">
+        <v>1441</v>
+      </c>
+      <c r="C11" s="142"/>
+      <c r="D11" s="142"/>
+      <c r="E11" s="142"/>
+      <c r="F11" s="142"/>
+      <c r="G11" s="142"/>
+      <c r="H11" s="142"/>
+      <c r="I11" s="127" t="s">
         <v>1442</v>
-      </c>
-      <c r="C11" s="135"/>
-      <c r="D11" s="135"/>
-      <c r="E11" s="135"/>
-      <c r="F11" s="135"/>
-      <c r="G11" s="135"/>
-      <c r="H11" s="135"/>
-      <c r="I11" s="127" t="s">
-        <v>1443</v>
       </c>
     </row>
     <row r="12" spans="1:9">
       <c r="A12" s="127" t="s">
         <v>931</v>
       </c>
-      <c r="B12" s="135" t="s">
+      <c r="B12" s="142" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C12" s="142"/>
+      <c r="D12" s="142"/>
+      <c r="E12" s="142"/>
+      <c r="F12" s="142"/>
+      <c r="G12" s="142"/>
+      <c r="H12" s="142"/>
+      <c r="I12" s="127" t="s">
         <v>1446</v>
-      </c>
-      <c r="C12" s="135"/>
-      <c r="D12" s="135"/>
-      <c r="E12" s="135"/>
-      <c r="F12" s="135"/>
-      <c r="G12" s="135"/>
-      <c r="H12" s="135"/>
-      <c r="I12" s="127" t="s">
-        <v>1447</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="15">
       <c r="A14" s="131" t="s">
-        <v>1448</v>
+        <v>1447</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -18657,28 +18524,28 @@
         <v>121</v>
       </c>
       <c r="B15" s="129" t="s">
+        <v>1448</v>
+      </c>
+      <c r="C15" s="129" t="s">
         <v>1449</v>
       </c>
-      <c r="C15" s="129" t="s">
+      <c r="D15" s="129" t="s">
         <v>1450</v>
       </c>
-      <c r="D15" s="129" t="s">
+      <c r="E15" s="129" t="s">
         <v>1451</v>
       </c>
-      <c r="E15" s="129" t="s">
+      <c r="F15" s="129" t="s">
         <v>1452</v>
       </c>
-      <c r="F15" s="129" t="s">
+      <c r="G15" s="129" t="s">
         <v>1453</v>
       </c>
-      <c r="G15" s="129" t="s">
+      <c r="H15" s="129" t="s">
         <v>1454</v>
       </c>
-      <c r="H15" s="129" t="s">
+      <c r="I15" s="129" t="s">
         <v>1455</v>
-      </c>
-      <c r="I15" s="129" t="s">
-        <v>1456</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -18718,7 +18585,7 @@
         <v>2</v>
       </c>
       <c r="B17" s="134" t="s">
-        <v>1457</v>
+        <v>1456</v>
       </c>
       <c r="C17" s="132">
         <v>4</v>
@@ -18750,7 +18617,7 @@
         <v>3</v>
       </c>
       <c r="B18" s="134" t="s">
-        <v>1458</v>
+        <v>1457</v>
       </c>
       <c r="C18" s="132">
         <v>5</v>
@@ -18782,7 +18649,7 @@
         <v>4</v>
       </c>
       <c r="B19" s="134" t="s">
-        <v>1459</v>
+        <v>1458</v>
       </c>
       <c r="C19" s="132">
         <v>5</v>
@@ -18811,37 +18678,37 @@
     </row>
     <row r="21" spans="1:9" ht="15">
       <c r="A21" s="99" t="s">
-        <v>1410</v>
+        <v>1409</v>
       </c>
     </row>
     <row r="22" spans="1:9">
       <c r="A22" s="127" t="s">
-        <v>1460</v>
+        <v>1459</v>
       </c>
     </row>
     <row r="23" spans="1:9">
       <c r="A23" s="127" t="s">
-        <v>1461</v>
+        <v>1460</v>
       </c>
     </row>
     <row r="24" spans="1:9">
       <c r="A24" s="127" t="s">
-        <v>1462</v>
+        <v>1461</v>
       </c>
     </row>
     <row r="25" spans="1:9">
       <c r="A25" s="127" t="s">
-        <v>1463</v>
+        <v>1462</v>
       </c>
     </row>
     <row r="26" spans="1:9">
       <c r="A26" s="127" t="s">
-        <v>1464</v>
+        <v>1463</v>
       </c>
     </row>
     <row r="27" spans="1:9">
       <c r="A27" s="127" t="s">
-        <v>1465</v>
+        <v>1464</v>
       </c>
     </row>
   </sheetData>
@@ -18930,7 +18797,7 @@
         <v>14</v>
       </c>
       <c r="C7" s="115" t="s">
-        <v>1483</v>
+        <v>1482</v>
       </c>
       <c r="D7" s="115" t="s">
         <v>1379</v>
@@ -19014,7 +18881,7 @@
         <v>35</v>
       </c>
       <c r="C13" s="115" t="s">
-        <v>1472</v>
+        <v>1471</v>
       </c>
       <c r="D13" s="115" t="s">
         <v>36</v>
@@ -19161,12 +19028,12 @@
     </row>
     <row r="46" spans="1:1">
       <c r="A46" s="123" t="s">
-        <v>1493</v>
+        <v>1492</v>
       </c>
     </row>
     <row r="47" spans="1:1">
       <c r="A47" s="123" t="s">
-        <v>1488</v>
+        <v>1487</v>
       </c>
     </row>
     <row r="48" spans="1:1">
@@ -21682,7 +21549,7 @@
         <v>충분</v>
       </c>
       <c r="F22" s="115" t="s">
-        <v>1478</v>
+        <v>1477</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="30" customHeight="1">
@@ -21912,7 +21779,7 @@
     </row>
     <row r="59" spans="1:1">
       <c r="A59" s="123" t="s">
-        <v>1479</v>
+        <v>1478</v>
       </c>
     </row>
     <row r="60" spans="1:1">

</xml_diff>

<commit_message>
운동프로그램 갱신 2026-10-05  4:43:12.91
</commit_message>
<xml_diff>
--- a/운동프로그램_주6회_v20.xlsx
+++ b/운동프로그램_주6회_v20.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b2bc197408547891/Desktop/운동/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="671" documentId="11_6AF0B42629B6F5CFF7DAC05DB27E968F34409905" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8E88B6C2-E753-46D1-AC6E-58733FDE3FBC}"/>
+  <xr:revisionPtr revIDLastSave="680" documentId="11_6AF0B42629B6F5CFF7DAC05DB27E968F34409905" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6C6281F1-095F-4AFD-A580-A2EC34C200D4}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="976" firstSheet="1" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="976" firstSheet="5" activeTab="25" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="시작중량_설정" sheetId="1" r:id="rId1"/>
@@ -12681,7 +12681,7 @@
       </c>
       <c r="E8" s="121">
         <f>복귀_월_가슴!$E$26</f>
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F8" s="114" t="s">
         <v>1373</v>
@@ -12705,7 +12705,7 @@
       </c>
       <c r="E9" s="121">
         <f>복귀_화_팔!$E$20</f>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F9" s="114" t="s">
         <v>1457</v>
@@ -12794,7 +12794,7 @@
       <c r="D13" s="122"/>
       <c r="E13" s="116">
         <f>SUM(E6:E12)</f>
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="F13" s="116" t="s">
         <v>1498</v>
@@ -14901,7 +14901,7 @@
         <v>30</v>
       </c>
       <c r="E25" s="114">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F25" s="114" t="s">
         <v>1350</v>
@@ -14914,7 +14914,7 @@
       </c>
       <c r="I25" s="114">
         <f>IF(E25=0,0,ROUND((E25*(G25+H25)+N25)/60,1))</f>
-        <v>3.3</v>
+        <v>6.7</v>
       </c>
       <c r="J25" s="115" t="s">
         <v>1365</v>
@@ -14935,14 +14935,14 @@
       </c>
       <c r="E26" s="116">
         <f>SUM(E18:E25)</f>
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F26" s="116"/>
       <c r="G26" s="116"/>
       <c r="H26" s="116"/>
       <c r="I26" s="116">
         <f>ROUND(SUM(I18:I25),0)</f>
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="28" spans="1:14">
@@ -15175,7 +15175,7 @@
         <v>6</v>
       </c>
       <c r="E12" s="114">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F12" s="114" t="s">
         <v>281</v>
@@ -15188,7 +15188,7 @@
       </c>
       <c r="I12" s="114">
         <f t="shared" si="0"/>
-        <v>5.8</v>
+        <v>7.7</v>
       </c>
       <c r="J12" s="115" t="s">
         <v>1086</v>
@@ -15486,14 +15486,14 @@
       </c>
       <c r="E20" s="116">
         <f>SUM(E11:E19)</f>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F20" s="116"/>
       <c r="G20" s="116"/>
       <c r="H20" s="116"/>
       <c r="I20" s="116">
         <f>ROUND(SUM(I11:I19),0)</f>
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="22" spans="1:14">
@@ -20329,11 +20329,11 @@
       </c>
       <c r="E45" s="114">
         <f t="shared" ca="1" si="4"/>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F45" s="114">
         <f t="shared" ref="F45" ca="1" si="6">IF(ISNUMBER(E45),$D45*E45,0)</f>
-        <v>0.66</v>
+        <v>1.32</v>
       </c>
       <c r="G45" s="114" t="s">
         <v>666</v>
@@ -20917,11 +20917,11 @@
       </c>
       <c r="E66" s="114">
         <f t="shared" ca="1" si="4"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F66" s="114">
         <f t="shared" ca="1" si="5"/>
-        <v>0.99</v>
+        <v>1.32</v>
       </c>
       <c r="G66" s="114" t="s">
         <v>666</v>
@@ -21287,7 +21287,7 @@
       </c>
       <c r="I7" s="125">
         <f ca="1">SUM(D7:D10)</f>
-        <v>49</v>
+        <v>49.5</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="30" customHeight="1">
@@ -21355,11 +21355,11 @@
       </c>
       <c r="C10" s="114">
         <f ca="1">MROUND(SUMIFS(복귀_간접계수맵!$F$7:$F$94,복귀_간접계수맵!$C$7:$C$94,$A10),0.5)</f>
-        <v>6</v>
+        <v>6.5</v>
       </c>
       <c r="D10" s="114">
         <f t="shared" ca="1" si="0"/>
-        <v>19</v>
+        <v>19.5</v>
       </c>
       <c r="E10" s="114" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -21447,7 +21447,7 @@
       </c>
       <c r="B14" s="114">
         <f>SUMIFS(복귀_토_하체전면!$E:$E,복귀_토_하체전면!$C:$C,$A14)+SUMIFS(복귀_일_수평당기기!$E:$E,복귀_일_수평당기기!$C:$C,$A14)+SUMIFS(복귀_월_가슴!$E:$E,복귀_월_가슴!$C:$C,$A14)+SUMIFS(복귀_화_팔!$E:$E,복귀_화_팔!$C:$C,$A14)+SUMIFS(복귀_수_하체후면!$E:$E,복귀_수_하체후면!$C:$C,$A14)+SUMIFS(복귀_목_수직당기기!$E:$E,복귀_목_수직당기기!$C:$C,$A14)</f>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C14" s="114">
         <f ca="1">MROUND(SUMIFS(복귀_간접계수맵!$F$7:$F$94,복귀_간접계수맵!$C$7:$C$94,$A14),0.5)</f>
@@ -21455,7 +21455,7 @@
       </c>
       <c r="D14" s="114">
         <f t="shared" ca="1" si="0"/>
-        <v>13.5</v>
+        <v>15.5</v>
       </c>
       <c r="E14" s="114" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -21598,7 +21598,7 @@
       </c>
       <c r="B20" s="114">
         <f>SUMIFS(복귀_토_하체전면!$E:$E,복귀_토_하체전면!$C:$C,$A20)+SUMIFS(복귀_일_수평당기기!$E:$E,복귀_일_수평당기기!$C:$C,$A20)+SUMIFS(복귀_월_가슴!$E:$E,복귀_월_가슴!$C:$C,$A20)+SUMIFS(복귀_화_팔!$E:$E,복귀_화_팔!$C:$C,$A20)+SUMIFS(복귀_수_하체후면!$E:$E,복귀_수_하체후면!$C:$C,$A20)+SUMIFS(복귀_목_수직당기기!$E:$E,복귀_목_수직당기기!$C:$C,$A20)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C20" s="114">
         <f ca="1">MROUND(SUMIFS(복귀_간접계수맵!$F$7:$F$94,복귀_간접계수맵!$C$7:$C$94,$A20),0.5)</f>
@@ -21606,7 +21606,7 @@
       </c>
       <c r="D20" s="114">
         <f t="shared" ca="1" si="0"/>
-        <v>16.5</v>
+        <v>17.5</v>
       </c>
       <c r="E20" s="114" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -21650,15 +21650,15 @@
       </c>
       <c r="C22" s="114">
         <f ca="1">MROUND(SUMIFS(복귀_간접계수맵!$F$7:$F$94,복귀_간접계수맵!$C$7:$C$94,$A22),0.5)</f>
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="D22" s="114">
         <f t="shared" ca="1" si="0"/>
-        <v>20</v>
+        <v>20.5</v>
       </c>
       <c r="E22" s="114" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>충분</v>
+        <v>과다 점검</v>
       </c>
       <c r="F22" s="115" t="s">
         <v>1466</v>
@@ -21742,11 +21742,11 @@
       </c>
       <c r="B26" s="116">
         <f>SUM(B5:B25)</f>
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="D26" s="116">
         <f ca="1">SUM(D5:D25)</f>
-        <v>269</v>
+        <v>273</v>
       </c>
     </row>
     <row r="28" spans="1:6">

</xml_diff>

<commit_message>
운동프로그램 갱신 2026-10-06  7:09:52.03
</commit_message>
<xml_diff>
--- a/운동프로그램_주6회_v20.xlsx
+++ b/운동프로그램_주6회_v20.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b2bc197408547891/Desktop/운동/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1745" documentId="11_6AF0B42629B6F5CFF7DAC05DB27E968F34409905" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{22418169-8B01-4FA1-8FF2-92C941176111}"/>
+  <xr:revisionPtr revIDLastSave="1746" documentId="11_6AF0B42629B6F5CFF7DAC05DB27E968F34409905" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C7E6D1B9-D4CC-412A-BE89-CDBA17F5A746}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="976" firstSheet="5" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1830" yWindow="1425" windowWidth="36435" windowHeight="19425" tabRatio="976" firstSheet="5" activeTab="17" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="시작중량_설정" sheetId="1" r:id="rId1"/>
@@ -12488,7 +12488,7 @@
       </c>
       <c r="E6" s="121">
         <f>복귀_토_하체전면!$E$31</f>
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F6" s="114" t="s">
         <v>1515</v>
@@ -12649,7 +12649,7 @@
       <c r="D13" s="122"/>
       <c r="E13" s="116">
         <f>SUM(E6:E12)</f>
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="F13" s="116" t="s">
         <v>1543</v>
@@ -13303,7 +13303,7 @@
         <v>30</v>
       </c>
       <c r="E23" s="114">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F23" s="114" t="s">
         <v>281</v>
@@ -13316,7 +13316,7 @@
       </c>
       <c r="I23" s="114">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>10.7</v>
       </c>
       <c r="J23" s="115" t="s">
         <v>988</v>
@@ -13620,14 +13620,14 @@
       </c>
       <c r="E31" s="116">
         <f>SUM(E20:E30)</f>
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F31" s="116"/>
       <c r="G31" s="116"/>
       <c r="H31" s="116"/>
       <c r="I31" s="116">
         <f>ROUND(SUM(I20:I30),0)</f>
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="33" spans="1:1">
@@ -20724,11 +20724,11 @@
       </c>
       <c r="E10" s="114">
         <f t="shared" ca="1" si="0"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F10" s="114">
         <f t="shared" ca="1" si="1"/>
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="G10" s="114" t="s">
         <v>666</v>
@@ -21340,11 +21340,11 @@
       </c>
       <c r="E32" s="114">
         <f t="shared" ca="1" si="0"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F32" s="114">
         <f t="shared" ca="1" si="1"/>
-        <v>0.99</v>
+        <v>1.32</v>
       </c>
       <c r="G32" s="114" t="s">
         <v>666</v>
@@ -22886,7 +22886,7 @@
       </c>
       <c r="B12" s="114">
         <f>SUMIFS(복귀_토_하체전면!$E:$E,복귀_토_하체전면!$C:$C,$A12)+SUMIFS(복귀_일_수평당기기!$E:$E,복귀_일_수평당기기!$C:$C,$A12)+SUMIFS(복귀_월_가슴!$E:$E,복귀_월_가슴!$C:$C,$A12)+SUMIFS(복귀_화_팔!$E:$E,복귀_화_팔!$C:$C,$A12)+SUMIFS(복귀_수_하체후면!$E:$E,복귀_수_하체후면!$C:$C,$A12)+SUMIFS(복귀_목_수직당기기!$E:$E,복귀_목_수직당기기!$C:$C,$A12)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C12" s="114">
         <f ca="1">MROUND(SUMIFS(복귀_간접계수맵!$F$7:$F$98,복귀_간접계수맵!$C$7:$C$98,$A12),0.5)</f>
@@ -22894,7 +22894,7 @@
       </c>
       <c r="D12" s="114">
         <f t="shared" ca="1" si="0"/>
-        <v>12.5</v>
+        <v>13.5</v>
       </c>
       <c r="E12" s="114" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -22914,11 +22914,11 @@
       </c>
       <c r="C13" s="114">
         <f ca="1">MROUND(SUMIFS(복귀_간접계수맵!$F$7:$F$98,복귀_간접계수맵!$C$7:$C$98,$A13),0.5)</f>
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="D13" s="114">
         <f t="shared" ca="1" si="0"/>
-        <v>21</v>
+        <v>21.5</v>
       </c>
       <c r="E13" s="114" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -23113,11 +23113,11 @@
       </c>
       <c r="C21" s="114">
         <f ca="1">MROUND(SUMIFS(복귀_간접계수맵!$F$7:$F$98,복귀_간접계수맵!$C$7:$C$98,$A21),0.5)</f>
-        <v>8.5</v>
+        <v>9</v>
       </c>
       <c r="D21" s="114">
         <f t="shared" ca="1" si="0"/>
-        <v>17.5</v>
+        <v>18</v>
       </c>
       <c r="E21" s="114" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -23229,11 +23229,11 @@
       </c>
       <c r="B26" s="116">
         <f>SUM(B5:B25)</f>
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D26" s="116">
         <f ca="1">SUM(D5:D25)</f>
-        <v>287.5</v>
+        <v>289.5</v>
       </c>
     </row>
     <row r="28" spans="1:6">

</xml_diff>